<commit_message>
feat(survey): yangi so'rovnoma ma'lumotlari kiritildi (Niyozova Komila, 26-03), davomat va hisobotlar yangilandi
</commit_message>
<xml_diff>
--- a/hisobotlar/1-kurs_Sorovnoma_Malumotlari.xlsx
+++ b/hisobotlar/1-kurs_Sorovnoma_Malumotlari.xlsx
@@ -4365,38 +4365,74 @@
       <c r="N59" s="13" t="inlineStr"/>
     </row>
     <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="10" t="n">
+      <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>26-03</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Niyozova Komila Toshpulatovna</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>To'ldirmagan</t>
-        </is>
-      </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>To'ldirgan</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>24.05.1983</t>
         </is>
       </c>
-      <c r="F60" s="13" t="inlineStr"/>
-      <c r="G60" s="13" t="inlineStr"/>
-      <c r="H60" s="13" t="inlineStr"/>
-      <c r="I60" s="13" t="inlineStr"/>
-      <c r="J60" s="13" t="inlineStr"/>
-      <c r="K60" s="10" t="inlineStr"/>
-      <c r="L60" s="10" t="inlineStr"/>
-      <c r="M60" s="10" t="inlineStr"/>
-      <c r="N60" s="13" t="inlineStr"/>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Kitob tumani</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Alaqo'yliq MFY</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Mevali ko'chasi</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>109-uy</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>Kitob tumani, Alaqo'yliq MFY, Mevali ko'chasi, 109-uy</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>O'z uyidan</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>+998 99 217-47-52</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>+998 95 528-40-81</t>
+        </is>
+      </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
+          <t>Turmush o'rtog'i</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="6" t="n">

</xml_diff>